<commit_message>
nang cap he thong lan 2
</commit_message>
<xml_diff>
--- a/game_theo_chu_de.xlsx
+++ b/game_theo_chu_de.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J306"/>
+  <dimension ref="A1:J315"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -800,7 +800,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B13" t="str">
-        <v>名字</v>
+        <v>们</v>
       </c>
       <c r="C13" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -832,7 +832,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B14" t="str">
-        <v>男</v>
+        <v>名字</v>
       </c>
       <c r="C14" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -864,7 +864,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B15" t="str">
-        <v>男朋友</v>
+        <v>男</v>
       </c>
       <c r="C15" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -896,7 +896,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B16" t="str">
-        <v>你</v>
+        <v>男朋友</v>
       </c>
       <c r="C16" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -928,7 +928,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B17" t="str">
-        <v>你们</v>
+        <v>你</v>
       </c>
       <c r="C17" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -960,7 +960,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B18" t="str">
-        <v>您</v>
+        <v>你们</v>
       </c>
       <c r="C18" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -992,7 +992,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B19" t="str">
-        <v>女</v>
+        <v>您</v>
       </c>
       <c r="C19" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1024,7 +1024,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B20" t="str">
-        <v>女儿</v>
+        <v>女</v>
       </c>
       <c r="C20" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1056,7 +1056,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B21" t="str">
-        <v>女朋友</v>
+        <v>女儿</v>
       </c>
       <c r="C21" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1088,7 +1088,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B22" t="str">
-        <v>女士</v>
+        <v>女朋友</v>
       </c>
       <c r="C22" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1120,7 +1120,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B23" t="str">
-        <v>朋友</v>
+        <v>女士</v>
       </c>
       <c r="C23" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1152,7 +1152,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B24" t="str">
-        <v>人</v>
+        <v>朋友</v>
       </c>
       <c r="C24" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1184,7 +1184,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B25" t="str">
-        <v>谁</v>
+        <v>人</v>
       </c>
       <c r="C25" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1216,7 +1216,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B26" t="str">
-        <v>他</v>
+        <v>谁</v>
       </c>
       <c r="C26" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1248,7 +1248,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B27" t="str">
-        <v>他们</v>
+        <v>他</v>
       </c>
       <c r="C27" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1280,7 +1280,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B28" t="str">
-        <v>它</v>
+        <v>他们</v>
       </c>
       <c r="C28" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1312,7 +1312,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B29" t="str">
-        <v>它们</v>
+        <v>它</v>
       </c>
       <c r="C29" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1344,7 +1344,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B30" t="str">
-        <v>她们</v>
+        <v>它们</v>
       </c>
       <c r="C30" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1376,7 +1376,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B31" t="str">
-        <v>同学</v>
+        <v>她们</v>
       </c>
       <c r="C31" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1408,7 +1408,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B32" t="str">
-        <v>我</v>
+        <v>同学</v>
       </c>
       <c r="C32" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1440,7 +1440,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B33" t="str">
-        <v>我们</v>
+        <v>我</v>
       </c>
       <c r="C33" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1472,7 +1472,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B34" t="str">
-        <v>先生</v>
+        <v>我们</v>
       </c>
       <c r="C34" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1504,7 +1504,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B35" t="str">
-        <v>小朋友</v>
+        <v>先生</v>
       </c>
       <c r="C35" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1536,7 +1536,7 @@
         <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B36" t="str">
-        <v>她</v>
+        <v>小朋友</v>
       </c>
       <c r="C36" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1565,10 +1565,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2. Cơ thể &amp; Sức khỏe</v>
+        <v>1. Con người &amp; Các mối quan hệ</v>
       </c>
       <c r="B37" t="str">
-        <v>病</v>
+        <v>她</v>
       </c>
       <c r="C37" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1600,7 +1600,7 @@
         <v>2. Cơ thể &amp; Sức khỏe</v>
       </c>
       <c r="B38" t="str">
-        <v>病人</v>
+        <v>病</v>
       </c>
       <c r="C38" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1632,7 +1632,7 @@
         <v>2. Cơ thể &amp; Sức khỏe</v>
       </c>
       <c r="B39" t="str">
-        <v>看病</v>
+        <v>病人</v>
       </c>
       <c r="C39" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1664,7 +1664,7 @@
         <v>2. Cơ thể &amp; Sức khỏe</v>
       </c>
       <c r="B40" t="str">
-        <v>生病</v>
+        <v>看病</v>
       </c>
       <c r="C40" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1696,7 +1696,7 @@
         <v>2. Cơ thể &amp; Sức khỏe</v>
       </c>
       <c r="B41" t="str">
-        <v>药</v>
+        <v>生病</v>
       </c>
       <c r="C41" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1725,10 +1725,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>3. Cảm xúc &amp; Thái độ</v>
+        <v>2. Cơ thể &amp; Sức khỏe</v>
       </c>
       <c r="B42" t="str">
-        <v>爱</v>
+        <v>药</v>
       </c>
       <c r="C42" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1760,7 +1760,7 @@
         <v>3. Cảm xúc &amp; Thái độ</v>
       </c>
       <c r="B43" t="str">
-        <v>高兴</v>
+        <v>爱</v>
       </c>
       <c r="C43" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1792,7 +1792,7 @@
         <v>3. Cảm xúc &amp; Thái độ</v>
       </c>
       <c r="B44" t="str">
-        <v>觉得</v>
+        <v>高兴</v>
       </c>
       <c r="C44" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1824,7 +1824,7 @@
         <v>3. Cảm xúc &amp; Thái độ</v>
       </c>
       <c r="B45" t="str">
-        <v>喜欢</v>
+        <v>觉得</v>
       </c>
       <c r="C45" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1853,10 +1853,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>4. Tư duy &amp; Nhận thức</v>
+        <v>3. Cảm xúc &amp; Thái độ</v>
       </c>
       <c r="B46" t="str">
-        <v>读</v>
+        <v>喜欢</v>
       </c>
       <c r="C46" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1888,7 +1888,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B47" t="str">
-        <v>读书</v>
+        <v>读</v>
       </c>
       <c r="C47" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1920,7 +1920,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B48" t="str">
-        <v>见</v>
+        <v>读书</v>
       </c>
       <c r="C48" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1952,7 +1952,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B49" t="str">
-        <v>叫</v>
+        <v>见</v>
       </c>
       <c r="C49" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -1984,7 +1984,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B50" t="str">
-        <v>看</v>
+        <v>叫</v>
       </c>
       <c r="C50" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2016,7 +2016,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B51" t="str">
-        <v>看见</v>
+        <v>看</v>
       </c>
       <c r="C51" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2048,7 +2048,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B52" t="str">
-        <v>请问</v>
+        <v>看见</v>
       </c>
       <c r="C52" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2080,7 +2080,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B53" t="str">
-        <v>认识</v>
+        <v>请问</v>
       </c>
       <c r="C53" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2112,7 +2112,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B54" t="str">
-        <v>说话</v>
+        <v>认识</v>
       </c>
       <c r="C54" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2144,7 +2144,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B55" t="str">
-        <v>听</v>
+        <v>说</v>
       </c>
       <c r="C55" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2176,7 +2176,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B56" t="str">
-        <v>听见</v>
+        <v>说话</v>
       </c>
       <c r="C56" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2208,7 +2208,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B57" t="str">
-        <v>问</v>
+        <v>听</v>
       </c>
       <c r="C57" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2240,7 +2240,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B58" t="str">
-        <v>问题</v>
+        <v>听见</v>
       </c>
       <c r="C58" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2272,7 +2272,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B59" t="str">
-        <v>想</v>
+        <v>问</v>
       </c>
       <c r="C59" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2304,7 +2304,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B60" t="str">
-        <v>学</v>
+        <v>问题</v>
       </c>
       <c r="C60" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2336,7 +2336,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B61" t="str">
-        <v>学习</v>
+        <v>想</v>
       </c>
       <c r="C61" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2368,7 +2368,7 @@
         <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B62" t="str">
-        <v>知道</v>
+        <v>学</v>
       </c>
       <c r="C62" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2397,10 +2397,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>5. Đời sống sinh hoạt</v>
+        <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B63" t="str">
-        <v>唱</v>
+        <v>学习</v>
       </c>
       <c r="C63" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2429,10 +2429,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>5. Đời sống sinh hoạt</v>
+        <v>4. Tư duy &amp; Nhận thức</v>
       </c>
       <c r="B64" t="str">
-        <v>吃</v>
+        <v>知道</v>
       </c>
       <c r="C64" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2464,7 +2464,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B65" t="str">
-        <v>穿</v>
+        <v>唱</v>
       </c>
       <c r="C65" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2496,7 +2496,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B66" t="str">
-        <v>打电话</v>
+        <v>吃</v>
       </c>
       <c r="C66" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2528,7 +2528,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B67" t="str">
-        <v>歌</v>
+        <v>穿</v>
       </c>
       <c r="C67" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2560,7 +2560,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B68" t="str">
-        <v>给</v>
+        <v>打电话</v>
       </c>
       <c r="C68" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2592,7 +2592,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B69" t="str">
-        <v>喝</v>
+        <v>歌</v>
       </c>
       <c r="C69" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2624,7 +2624,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B70" t="str">
-        <v>开</v>
+        <v>给</v>
       </c>
       <c r="C70" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2656,7 +2656,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B71" t="str">
-        <v>買</v>
+        <v>喝</v>
       </c>
       <c r="C71" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2688,7 +2688,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B72" t="str">
-        <v>卖</v>
+        <v>开</v>
       </c>
       <c r="C72" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2720,7 +2720,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B73" t="str">
-        <v>起床</v>
+        <v>买</v>
       </c>
       <c r="C73" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2752,7 +2752,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B74" t="str">
-        <v>玩</v>
+        <v>卖</v>
       </c>
       <c r="C74" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2784,7 +2784,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B75" t="str">
-        <v>写</v>
+        <v>起床</v>
       </c>
       <c r="C75" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2816,7 +2816,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B76" t="str">
-        <v>休息</v>
+        <v>睡</v>
       </c>
       <c r="C76" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2848,7 +2848,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B77" t="str">
-        <v>找</v>
+        <v>睡觉</v>
       </c>
       <c r="C77" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2880,7 +2880,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B78" t="str">
-        <v>住</v>
+        <v>玩</v>
       </c>
       <c r="C78" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2912,7 +2912,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B79" t="str">
-        <v>做</v>
+        <v>写</v>
       </c>
       <c r="C79" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2944,7 +2944,7 @@
         <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B80" t="str">
-        <v>做饭</v>
+        <v>休息</v>
       </c>
       <c r="C80" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -2973,10 +2973,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>6. Đồ vật &amp; Công cụ</v>
+        <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B81" t="str">
-        <v>杯</v>
+        <v>找</v>
       </c>
       <c r="C81" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3005,10 +3005,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>6. Đồ vật &amp; Công cụ</v>
+        <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B82" t="str">
-        <v>杯子</v>
+        <v>住</v>
       </c>
       <c r="C82" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3037,10 +3037,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>6. Đồ vật &amp; Công cụ</v>
+        <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B83" t="str">
-        <v>电话</v>
+        <v>做</v>
       </c>
       <c r="C83" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>6. Đồ vật &amp; Công cụ</v>
+        <v>5. Đời sống sinh hoạt</v>
       </c>
       <c r="B84" t="str">
-        <v>电脑</v>
+        <v>做饭</v>
       </c>
       <c r="C84" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3104,7 +3104,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B85" t="str">
-        <v>电视</v>
+        <v>杯</v>
       </c>
       <c r="C85" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3136,7 +3136,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B86" t="str">
-        <v>电影</v>
+        <v>杯子</v>
       </c>
       <c r="C86" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3168,7 +3168,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B87" t="str">
-        <v>东西</v>
+        <v>电话</v>
       </c>
       <c r="C87" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3200,7 +3200,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B88" t="str">
-        <v>件</v>
+        <v>电脑</v>
       </c>
       <c r="C88" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3232,7 +3232,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B89" t="str">
-        <v>钱</v>
+        <v>电视</v>
       </c>
       <c r="C89" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3264,7 +3264,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B90" t="str">
-        <v>事</v>
+        <v>电影</v>
       </c>
       <c r="C90" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3296,7 +3296,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B91" t="str">
-        <v>手机</v>
+        <v>东西</v>
       </c>
       <c r="C91" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3328,7 +3328,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B92" t="str">
-        <v>书</v>
+        <v>件</v>
       </c>
       <c r="C92" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3360,7 +3360,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B93" t="str">
-        <v>衣服</v>
+        <v>钱</v>
       </c>
       <c r="C93" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3392,7 +3392,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B94" t="str">
-        <v>椅子</v>
+        <v>事</v>
       </c>
       <c r="C94" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3424,7 +3424,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B95" t="str">
-        <v>元</v>
+        <v>手机</v>
       </c>
       <c r="C95" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3456,7 +3456,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B96" t="str">
-        <v>中文</v>
+        <v>书</v>
       </c>
       <c r="C96" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3488,7 +3488,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B97" t="str">
-        <v>桌子</v>
+        <v>衣服</v>
       </c>
       <c r="C97" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3520,7 +3520,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B98" t="str">
-        <v>字</v>
+        <v>椅子</v>
       </c>
       <c r="C98" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3552,7 +3552,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B99" t="str">
-        <v>汉语</v>
+        <v>元</v>
       </c>
       <c r="C99" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3584,7 +3584,7 @@
         <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B100" t="str">
-        <v>汉字</v>
+        <v>中文</v>
       </c>
       <c r="C100" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3613,10 +3613,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>7. Địa điểm &amp; Nơi chốn</v>
+        <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B101" t="str">
-        <v>超市</v>
+        <v>桌子</v>
       </c>
       <c r="C101" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3645,10 +3645,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>7. Địa điểm &amp; Nơi chốn</v>
+        <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B102" t="str">
-        <v>大学</v>
+        <v>字</v>
       </c>
       <c r="C102" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3677,10 +3677,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>7. Địa điểm &amp; Nơi chốn</v>
+        <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B103" t="str">
-        <v>电影院</v>
+        <v>汉语</v>
       </c>
       <c r="C103" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3709,10 +3709,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>7. Địa điểm &amp; Nơi chốn</v>
+        <v>6. Đồ vật &amp; Công cụ</v>
       </c>
       <c r="B104" t="str">
-        <v>店</v>
+        <v>汉字</v>
       </c>
       <c r="C104" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3744,7 +3744,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B105" t="str">
-        <v>饭店</v>
+        <v>超市</v>
       </c>
       <c r="C105" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3776,7 +3776,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B106" t="str">
-        <v>房间</v>
+        <v>大学</v>
       </c>
       <c r="C106" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3808,7 +3808,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B107" t="str">
-        <v>公司</v>
+        <v>电影院</v>
       </c>
       <c r="C107" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3840,7 +3840,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B108" t="str">
-        <v>狗</v>
+        <v>店</v>
       </c>
       <c r="C108" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3872,7 +3872,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B109" t="str">
-        <v>国</v>
+        <v>饭店</v>
       </c>
       <c r="C109" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3904,7 +3904,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B110" t="str">
-        <v>机场</v>
+        <v>房间</v>
       </c>
       <c r="C110" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3936,7 +3936,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B111" t="str">
-        <v>家</v>
+        <v>公司</v>
       </c>
       <c r="C111" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -3968,7 +3968,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B112" t="str">
-        <v>哪</v>
+        <v>国</v>
       </c>
       <c r="C112" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4000,7 +4000,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B113" t="str">
-        <v>哪儿</v>
+        <v>机场</v>
       </c>
       <c r="C113" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4032,7 +4032,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B114" t="str">
-        <v>那里</v>
+        <v>家</v>
       </c>
       <c r="C114" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4064,7 +4064,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B115" t="str">
-        <v>那儿</v>
+        <v>哪</v>
       </c>
       <c r="C115" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4096,7 +4096,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B116" t="str">
-        <v>商店</v>
+        <v>哪儿</v>
       </c>
       <c r="C116" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4128,7 +4128,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B117" t="str">
-        <v>书店</v>
+        <v>那里</v>
       </c>
       <c r="C117" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4160,7 +4160,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B118" t="str">
-        <v>小学</v>
+        <v>那儿</v>
       </c>
       <c r="C118" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4192,7 +4192,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B119" t="str">
-        <v>学校</v>
+        <v>商店</v>
       </c>
       <c r="C119" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4224,7 +4224,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B120" t="str">
-        <v>医院</v>
+        <v>书店</v>
       </c>
       <c r="C120" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4256,7 +4256,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B121" t="str">
-        <v>中国</v>
+        <v>小学</v>
       </c>
       <c r="C121" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4288,7 +4288,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B122" t="str">
-        <v>法国</v>
+        <v>学校</v>
       </c>
       <c r="C122" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4320,7 +4320,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B123" t="str">
-        <v>泰国</v>
+        <v>医院</v>
       </c>
       <c r="C123" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4352,7 +4352,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B124" t="str">
-        <v>这里</v>
+        <v>中国</v>
       </c>
       <c r="C124" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4384,7 +4384,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B125" t="str">
-        <v>这儿</v>
+        <v>法国</v>
       </c>
       <c r="C125" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4416,7 +4416,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B126" t="str">
-        <v>中学</v>
+        <v>泰国</v>
       </c>
       <c r="C126" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4448,7 +4448,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B127" t="str">
-        <v>西安</v>
+        <v>这里</v>
       </c>
       <c r="C127" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4480,7 +4480,7 @@
         <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B128" t="str">
-        <v>北京</v>
+        <v>这儿</v>
       </c>
       <c r="C128" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4509,10 +4509,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>8. Giao thông &amp; Di chuyển</v>
+        <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B129" t="str">
-        <v>车</v>
+        <v>中学</v>
       </c>
       <c r="C129" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4541,10 +4541,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>8. Giao thông &amp; Di chuyển</v>
+        <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B130" t="str">
-        <v>出租车</v>
+        <v>西安</v>
       </c>
       <c r="C130" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4573,10 +4573,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>8. Giao thông &amp; Di chuyển</v>
+        <v>7. Địa điểm &amp; Nơi chốn</v>
       </c>
       <c r="B131" t="str">
-        <v>到</v>
+        <v>北京</v>
       </c>
       <c r="C131" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4608,7 +4608,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B132" t="str">
-        <v>飞机</v>
+        <v>车</v>
       </c>
       <c r="C132" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4640,7 +4640,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B133" t="str">
-        <v>回</v>
+        <v>出租车</v>
       </c>
       <c r="C133" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4672,7 +4672,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B134" t="str">
-        <v>火车</v>
+        <v>到</v>
       </c>
       <c r="C134" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4704,7 +4704,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B135" t="str">
-        <v>开车</v>
+        <v>飞机</v>
       </c>
       <c r="C135" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4736,7 +4736,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B136" t="str">
-        <v>来</v>
+        <v>回</v>
       </c>
       <c r="C136" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4768,7 +4768,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B137" t="str">
-        <v>去</v>
+        <v>火车</v>
       </c>
       <c r="C137" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4800,7 +4800,7 @@
         <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B138" t="str">
-        <v>坐</v>
+        <v>开车</v>
       </c>
       <c r="C138" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4829,10 +4829,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>9. Không gian &amp; Vị trí</v>
+        <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B139" t="str">
-        <v>边</v>
+        <v>来</v>
       </c>
       <c r="C139" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4861,10 +4861,10 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>9. Không gian &amp; Vị trí</v>
+        <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B140" t="str">
-        <v>后</v>
+        <v>去</v>
       </c>
       <c r="C140" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4893,10 +4893,10 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>9. Không gian &amp; Vị trí</v>
+        <v>8. Giao thông &amp; Di chuyển</v>
       </c>
       <c r="B141" t="str">
-        <v>里</v>
+        <v>坐</v>
       </c>
       <c r="C141" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4928,7 +4928,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B142" t="str">
-        <v>哪里</v>
+        <v>边</v>
       </c>
       <c r="C142" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4960,7 +4960,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B143" t="str">
-        <v>那边</v>
+        <v>后</v>
       </c>
       <c r="C143" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -4992,7 +4992,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B144" t="str">
-        <v>那个</v>
+        <v>里</v>
       </c>
       <c r="C144" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5024,7 +5024,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B145" t="str">
-        <v>前</v>
+        <v>哪里</v>
       </c>
       <c r="C145" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5056,7 +5056,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B146" t="str">
-        <v>前边</v>
+        <v>那边</v>
       </c>
       <c r="C146" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5088,7 +5088,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B147" t="str">
-        <v>上</v>
+        <v>那个</v>
       </c>
       <c r="C147" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5120,7 +5120,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B148" t="str">
-        <v>外</v>
+        <v>前</v>
       </c>
       <c r="C148" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5152,7 +5152,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B149" t="str">
-        <v>外边</v>
+        <v>前边</v>
       </c>
       <c r="C149" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5184,7 +5184,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B150" t="str">
-        <v>下</v>
+        <v>上</v>
       </c>
       <c r="C150" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5216,7 +5216,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B151" t="str">
-        <v>这边</v>
+        <v>外</v>
       </c>
       <c r="C151" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5248,7 +5248,7 @@
         <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B152" t="str">
-        <v>这个</v>
+        <v>外边</v>
       </c>
       <c r="C152" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5277,10 +5277,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>10. Thời gian</v>
+        <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B153" t="str">
-        <v>白天</v>
+        <v>下</v>
       </c>
       <c r="C153" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5309,10 +5309,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>10. Thời gian</v>
+        <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B154" t="str">
-        <v>点</v>
+        <v>这边</v>
       </c>
       <c r="C154" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5341,10 +5341,10 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>10. Thời gian</v>
+        <v>9. Không gian &amp; Vị trí</v>
       </c>
       <c r="B155" t="str">
-        <v>分</v>
+        <v>这个</v>
       </c>
       <c r="C155" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5376,7 +5376,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B156" t="str">
-        <v>分钟</v>
+        <v>白天</v>
       </c>
       <c r="C156" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5408,7 +5408,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B157" t="str">
-        <v>今天</v>
+        <v>点</v>
       </c>
       <c r="C157" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5440,7 +5440,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B158" t="str">
-        <v>明年</v>
+        <v>分</v>
       </c>
       <c r="C158" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5472,7 +5472,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B159" t="str">
-        <v>明天</v>
+        <v>分钟</v>
       </c>
       <c r="C159" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5504,7 +5504,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B160" t="str">
-        <v>年</v>
+        <v>今年</v>
       </c>
       <c r="C160" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5536,7 +5536,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B161" t="str">
-        <v>去年</v>
+        <v>今天</v>
       </c>
       <c r="C161" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5568,7 +5568,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B162" t="str">
-        <v>日</v>
+        <v>明年</v>
       </c>
       <c r="C162" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5600,7 +5600,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B163" t="str">
-        <v>上午</v>
+        <v>明天</v>
       </c>
       <c r="C163" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5632,7 +5632,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B164" t="str">
-        <v>时候</v>
+        <v>年</v>
       </c>
       <c r="C164" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5664,7 +5664,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B165" t="str">
-        <v>时间</v>
+        <v>去年</v>
       </c>
       <c r="C165" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5696,7 +5696,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B166" t="str">
-        <v>晚</v>
+        <v>日</v>
       </c>
       <c r="C166" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5728,7 +5728,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B167" t="str">
-        <v>晚上</v>
+        <v>上午</v>
       </c>
       <c r="C167" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5760,7 +5760,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B168" t="str">
-        <v>下午</v>
+        <v>时候</v>
       </c>
       <c r="C168" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5792,7 +5792,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B169" t="str">
-        <v>现在</v>
+        <v>时间</v>
       </c>
       <c r="C169" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5824,7 +5824,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B170" t="str">
-        <v>小时</v>
+        <v>晚</v>
       </c>
       <c r="C170" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5856,7 +5856,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B171" t="str">
-        <v>星期</v>
+        <v>晚上</v>
       </c>
       <c r="C171" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5888,7 +5888,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B172" t="str">
-        <v>星期日</v>
+        <v>下午</v>
       </c>
       <c r="C172" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5920,7 +5920,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B173" t="str">
-        <v>星期天</v>
+        <v>现在</v>
       </c>
       <c r="C173" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5952,7 +5952,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B174" t="str">
-        <v>月</v>
+        <v>小时</v>
       </c>
       <c r="C174" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -5984,7 +5984,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B175" t="str">
-        <v>早</v>
+        <v>星期</v>
       </c>
       <c r="C175" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6016,7 +6016,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B176" t="str">
-        <v>中午</v>
+        <v>星期日</v>
       </c>
       <c r="C176" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6048,7 +6048,7 @@
         <v>10. Thời gian</v>
       </c>
       <c r="B177" t="str">
-        <v>昨天</v>
+        <v>星期天</v>
       </c>
       <c r="C177" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6077,10 +6077,10 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>11. Công việc &amp; Nghề nghiệp</v>
+        <v>10. Thời gian</v>
       </c>
       <c r="B178" t="str">
-        <v>大学生</v>
+        <v>月</v>
       </c>
       <c r="C178" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6109,10 +6109,10 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>11. Công việc &amp; Nghề nghiệp</v>
+        <v>10. Thời gian</v>
       </c>
       <c r="B179" t="str">
-        <v>服务员</v>
+        <v>早</v>
       </c>
       <c r="C179" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6141,10 +6141,10 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>11. Công việc &amp; Nghề nghiệp</v>
+        <v>10. Thời gian</v>
       </c>
       <c r="B180" t="str">
-        <v>工作</v>
+        <v>中午</v>
       </c>
       <c r="C180" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6173,10 +6173,10 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>11. Công việc &amp; Nghề nghiệp</v>
+        <v>10. Thời gian</v>
       </c>
       <c r="B181" t="str">
-        <v>老师</v>
+        <v>昨天</v>
       </c>
       <c r="C181" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6208,7 +6208,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B182" t="str">
-        <v>上班</v>
+        <v>大学生</v>
       </c>
       <c r="C182" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6240,7 +6240,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B183" t="str">
-        <v>上课</v>
+        <v>服务员</v>
       </c>
       <c r="C183" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6272,7 +6272,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B184" t="str">
-        <v>上学</v>
+        <v>工作</v>
       </c>
       <c r="C184" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6304,7 +6304,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B185" t="str">
-        <v>售货员</v>
+        <v>老师</v>
       </c>
       <c r="C185" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6336,7 +6336,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B186" t="str">
-        <v>下课</v>
+        <v>上班</v>
       </c>
       <c r="C186" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6368,7 +6368,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B187" t="str">
-        <v>小学生</v>
+        <v>上课</v>
       </c>
       <c r="C187" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6400,7 +6400,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B188" t="str">
-        <v>学生</v>
+        <v>上学</v>
       </c>
       <c r="C188" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6432,7 +6432,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B189" t="str">
-        <v>医</v>
+        <v>售货员</v>
       </c>
       <c r="C189" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6464,7 +6464,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B190" t="str">
-        <v>医生</v>
+        <v>下班</v>
       </c>
       <c r="C190" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6496,7 +6496,7 @@
         <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B191" t="str">
-        <v>中学生</v>
+        <v>下课</v>
       </c>
       <c r="C191" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6525,10 +6525,10 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>12. Miêu tả &amp; Đánh giá</v>
+        <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B192" t="str">
-        <v>大</v>
+        <v>小学生</v>
       </c>
       <c r="C192" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6557,10 +6557,10 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>12. Miêu tả &amp; Đánh giá</v>
+        <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B193" t="str">
-        <v>对</v>
+        <v>学生</v>
       </c>
       <c r="C193" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6589,10 +6589,10 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>12. Miêu tả &amp; Đánh giá</v>
+        <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B194" t="str">
-        <v>多</v>
+        <v>医</v>
       </c>
       <c r="C194" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6621,10 +6621,10 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>12. Miêu tả &amp; Đánh giá</v>
+        <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B195" t="str">
-        <v>非常</v>
+        <v>医生</v>
       </c>
       <c r="C195" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6653,10 +6653,10 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>12. Miêu tả &amp; Đánh giá</v>
+        <v>11. Công việc &amp; Nghề nghiệp</v>
       </c>
       <c r="B196" t="str">
-        <v>贵</v>
+        <v>中学生</v>
       </c>
       <c r="C196" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6688,7 +6688,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B197" t="str">
-        <v>好</v>
+        <v>大</v>
       </c>
       <c r="C197" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6720,7 +6720,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B198" t="str">
-        <v>好看</v>
+        <v>对</v>
       </c>
       <c r="C198" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6752,7 +6752,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B199" t="str">
-        <v>好听</v>
+        <v>多</v>
       </c>
       <c r="C199" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6784,7 +6784,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B200" t="str">
-        <v>好玩儿</v>
+        <v>非常</v>
       </c>
       <c r="C200" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6816,7 +6816,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B201" t="str">
-        <v>冷</v>
+        <v>贵</v>
       </c>
       <c r="C201" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6848,7 +6848,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B202" t="str">
-        <v>忙</v>
+        <v>好</v>
       </c>
       <c r="C202" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6880,7 +6880,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B203" t="str">
-        <v>便宜</v>
+        <v>好看</v>
       </c>
       <c r="C203" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6912,7 +6912,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B204" t="str">
-        <v>漂亮</v>
+        <v>好听</v>
       </c>
       <c r="C204" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6944,7 +6944,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B205" t="str">
-        <v>热</v>
+        <v>好玩儿</v>
       </c>
       <c r="C205" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -6976,7 +6976,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B206" t="str">
-        <v>少</v>
+        <v>冷</v>
       </c>
       <c r="C206" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7008,7 +7008,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B207" t="str">
-        <v>小</v>
+        <v>忙</v>
       </c>
       <c r="C207" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7040,7 +7040,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B208" t="str">
-        <v>新</v>
+        <v>便宜</v>
       </c>
       <c r="C208" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7072,7 +7072,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B209" t="str">
-        <v>真</v>
+        <v>漂亮</v>
       </c>
       <c r="C209" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7104,7 +7104,7 @@
         <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B210" t="str">
-        <v>正在</v>
+        <v>热</v>
       </c>
       <c r="C210" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7133,10 +7133,10 @@
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>13. Số lượng &amp; Đo lường</v>
+        <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B211" t="str">
-        <v>八</v>
+        <v>少</v>
       </c>
       <c r="C211" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7165,10 +7165,10 @@
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>13. Số lượng &amp; Đo lường</v>
+        <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B212" t="str">
-        <v>百</v>
+        <v>小</v>
       </c>
       <c r="C212" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7197,10 +7197,10 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>13. Số lượng &amp; Đo lường</v>
+        <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B213" t="str">
-        <v>半</v>
+        <v>新</v>
       </c>
       <c r="C213" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7229,10 +7229,10 @@
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>13. Số lượng &amp; Đo lường</v>
+        <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B214" t="str">
-        <v>本</v>
+        <v>真</v>
       </c>
       <c r="C214" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7261,10 +7261,10 @@
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>13. Số lượng &amp; Đo lường</v>
+        <v>12. Miêu tả &amp; Đánh giá</v>
       </c>
       <c r="B215" t="str">
-        <v>第</v>
+        <v>正在</v>
       </c>
       <c r="C215" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7296,7 +7296,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B216" t="str">
-        <v>多少</v>
+        <v>八</v>
       </c>
       <c r="C216" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7328,7 +7328,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B217" t="str">
-        <v>二</v>
+        <v>百</v>
       </c>
       <c r="C217" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7360,7 +7360,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B218" t="str">
-        <v>个</v>
+        <v>半</v>
       </c>
       <c r="C218" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7392,7 +7392,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B219" t="str">
-        <v>号</v>
+        <v>本</v>
       </c>
       <c r="C219" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7424,7 +7424,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B220" t="str">
-        <v>几</v>
+        <v>第</v>
       </c>
       <c r="C220" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7456,7 +7456,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B221" t="str">
-        <v>斤</v>
+        <v>多少</v>
       </c>
       <c r="C221" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7488,7 +7488,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B222" t="str">
-        <v>九</v>
+        <v>二</v>
       </c>
       <c r="C222" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7520,7 +7520,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B223" t="str">
-        <v>口</v>
+        <v>个</v>
       </c>
       <c r="C223" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7552,7 +7552,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B224" t="str">
-        <v>块</v>
+        <v>号</v>
       </c>
       <c r="C224" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7584,7 +7584,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B225" t="str">
-        <v>两</v>
+        <v>几</v>
       </c>
       <c r="C225" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7616,7 +7616,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B226" t="str">
-        <v>零</v>
+        <v>斤</v>
       </c>
       <c r="C226" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7648,7 +7648,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B227" t="str">
-        <v>六</v>
+        <v>九</v>
       </c>
       <c r="C227" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7680,7 +7680,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B228" t="str">
-        <v>七</v>
+        <v>口</v>
       </c>
       <c r="C228" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7712,7 +7712,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B229" t="str">
-        <v>千</v>
+        <v>块</v>
       </c>
       <c r="C229" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7744,7 +7744,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B230" t="str">
-        <v>三</v>
+        <v>两</v>
       </c>
       <c r="C230" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7776,7 +7776,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B231" t="str">
-        <v>十</v>
+        <v>零</v>
       </c>
       <c r="C231" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7808,7 +7808,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B232" t="str">
-        <v>四</v>
+        <v>六</v>
       </c>
       <c r="C232" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7840,7 +7840,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B233" t="str">
-        <v>岁</v>
+        <v>七</v>
       </c>
       <c r="C233" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7872,7 +7872,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B234" t="str">
-        <v>五</v>
+        <v>千</v>
       </c>
       <c r="C234" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7904,7 +7904,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B235" t="str">
-        <v>些</v>
+        <v>三</v>
       </c>
       <c r="C235" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7936,7 +7936,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B236" t="str">
-        <v>一</v>
+        <v>十</v>
       </c>
       <c r="C236" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -7968,7 +7968,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B237" t="str">
-        <v>一半</v>
+        <v>四</v>
       </c>
       <c r="C237" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8000,7 +8000,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B238" t="str">
-        <v>一下</v>
+        <v>岁</v>
       </c>
       <c r="C238" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8032,7 +8032,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B239" t="str">
-        <v>一点儿</v>
+        <v>五</v>
       </c>
       <c r="C239" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8064,7 +8064,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B240" t="str">
-        <v>一些</v>
+        <v>些</v>
       </c>
       <c r="C240" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8096,7 +8096,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B241" t="str">
-        <v>有</v>
+        <v>一</v>
       </c>
       <c r="C241" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8128,7 +8128,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B242" t="str">
-        <v>有的</v>
+        <v>一半</v>
       </c>
       <c r="C242" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8160,7 +8160,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B243" t="str">
-        <v>有点儿</v>
+        <v>一下</v>
       </c>
       <c r="C243" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8192,7 +8192,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B244" t="str">
-        <v>有些</v>
+        <v>一点儿</v>
       </c>
       <c r="C244" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8224,7 +8224,7 @@
         <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B245" t="str">
-        <v>只</v>
+        <v>一些</v>
       </c>
       <c r="C245" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8253,10 +8253,10 @@
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
+        <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B246" t="str">
-        <v>吧</v>
+        <v>有</v>
       </c>
       <c r="C246" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8285,10 +8285,10 @@
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
+        <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B247" t="str">
-        <v>不客气</v>
+        <v>有的</v>
       </c>
       <c r="C247" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8317,10 +8317,10 @@
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
+        <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B248" t="str">
-        <v>不要</v>
+        <v>有点儿</v>
       </c>
       <c r="C248" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8349,10 +8349,10 @@
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
+        <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B249" t="str">
-        <v>不</v>
+        <v>有些</v>
       </c>
       <c r="C249" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8381,10 +8381,10 @@
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
+        <v>13. Số lượng &amp; Đo lường</v>
       </c>
       <c r="B250" t="str">
-        <v>的</v>
+        <v>只</v>
       </c>
       <c r="C250" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8416,7 +8416,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B251" t="str">
-        <v>都</v>
+        <v>吧</v>
       </c>
       <c r="C251" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8448,7 +8448,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B252" t="str">
-        <v>对不起</v>
+        <v>不客气</v>
       </c>
       <c r="C252" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8480,7 +8480,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B253" t="str">
-        <v>还</v>
+        <v>不要</v>
       </c>
       <c r="C253" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8512,7 +8512,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B254" t="str">
-        <v>和</v>
+        <v>不</v>
       </c>
       <c r="C254" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8544,7 +8544,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B255" t="str">
-        <v>很</v>
+        <v>的</v>
       </c>
       <c r="C255" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8576,7 +8576,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B256" t="str">
-        <v>会</v>
+        <v>都</v>
       </c>
       <c r="C256" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8608,7 +8608,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B257" t="str">
-        <v>可以</v>
+        <v>对不起</v>
       </c>
       <c r="C257" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8640,7 +8640,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B258" t="str">
-        <v>了</v>
+        <v>还</v>
       </c>
       <c r="C258" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8672,7 +8672,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B259" t="str">
-        <v>吗</v>
+        <v>和</v>
       </c>
       <c r="C259" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8704,7 +8704,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B260" t="str">
-        <v>没</v>
+        <v>很</v>
       </c>
       <c r="C260" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8736,7 +8736,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B261" t="str">
-        <v>没关系</v>
+        <v>会</v>
       </c>
       <c r="C261" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8768,7 +8768,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B262" t="str">
-        <v>没事</v>
+        <v>可以</v>
       </c>
       <c r="C262" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8800,7 +8800,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B263" t="str">
-        <v>没有</v>
+        <v>了</v>
       </c>
       <c r="C263" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8832,7 +8832,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B264" t="str">
-        <v>那</v>
+        <v>吗</v>
       </c>
       <c r="C264" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8864,7 +8864,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B265" t="str">
-        <v>那些</v>
+        <v>没</v>
       </c>
       <c r="C265" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8896,7 +8896,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B266" t="str">
-        <v>呢</v>
+        <v>没关系</v>
       </c>
       <c r="C266" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8928,7 +8928,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B267" t="str">
-        <v>能</v>
+        <v>没事</v>
       </c>
       <c r="C267" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8960,7 +8960,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B268" t="str">
-        <v>你好</v>
+        <v>没有</v>
       </c>
       <c r="C268" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -8992,7 +8992,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B269" t="str">
-        <v>请</v>
+        <v>哪个</v>
       </c>
       <c r="C269" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9024,7 +9024,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B270" t="str">
-        <v>什么</v>
+        <v>哪些</v>
       </c>
       <c r="C270" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9056,7 +9056,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B271" t="str">
-        <v>是</v>
+        <v>那</v>
       </c>
       <c r="C271" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9088,7 +9088,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B272" t="str">
-        <v>太</v>
+        <v>那些</v>
       </c>
       <c r="C272" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9120,7 +9120,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B273" t="str">
-        <v>喂</v>
+        <v>呢</v>
       </c>
       <c r="C273" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9152,7 +9152,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B274" t="str">
-        <v>谢谢</v>
+        <v>能</v>
       </c>
       <c r="C274" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9184,7 +9184,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B275" t="str">
-        <v>要</v>
+        <v>你好</v>
       </c>
       <c r="C275" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9216,7 +9216,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B276" t="str">
-        <v>也</v>
+        <v>请</v>
       </c>
       <c r="C276" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9248,7 +9248,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B277" t="str">
-        <v>再</v>
+        <v>什么</v>
       </c>
       <c r="C277" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9280,7 +9280,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B278" t="str">
-        <v>再见</v>
+        <v>是</v>
       </c>
       <c r="C278" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9312,7 +9312,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B279" t="str">
-        <v>在大</v>
+        <v>太</v>
       </c>
       <c r="C279" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9344,7 +9344,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B280" t="str">
-        <v>怎么</v>
+        <v>喂</v>
       </c>
       <c r="C280" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9376,7 +9376,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B281" t="str">
-        <v>怎么样</v>
+        <v>谢谢</v>
       </c>
       <c r="C281" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9408,7 +9408,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B282" t="str">
-        <v>这</v>
+        <v>要</v>
       </c>
       <c r="C282" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9440,7 +9440,7 @@
         <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B283" t="str">
-        <v>这些</v>
+        <v>也</v>
       </c>
       <c r="C283" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9469,10 +9469,10 @@
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B284" t="str">
-        <v>猫</v>
+        <v>再</v>
       </c>
       <c r="C284" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9501,10 +9501,10 @@
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B285" t="str">
-        <v>水</v>
+        <v>再见</v>
       </c>
       <c r="C285" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9533,10 +9533,10 @@
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B286" t="str">
-        <v>天</v>
+        <v>在</v>
       </c>
       <c r="C286" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9565,10 +9565,10 @@
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B287" t="str">
-        <v>天气</v>
+        <v>怎么</v>
       </c>
       <c r="C287" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9597,10 +9597,10 @@
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B288" t="str">
-        <v>下雨</v>
+        <v>怎么样</v>
       </c>
       <c r="C288" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9629,10 +9629,10 @@
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B289" t="str">
-        <v>雪</v>
+        <v>这</v>
       </c>
       <c r="C289" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9661,10 +9661,10 @@
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>15. Tự nhiên</v>
+        <v>14. Công cụ ngữ pháp &amp; Cấu trúc</v>
       </c>
       <c r="B290" t="str">
-        <v>雨</v>
+        <v>这些</v>
       </c>
       <c r="C290" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9696,7 +9696,7 @@
         <v>15. Tự nhiên</v>
       </c>
       <c r="B291" t="str">
-        <v>早上</v>
+        <v>狗</v>
       </c>
       <c r="C291" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9725,10 +9725,10 @@
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B292" t="str">
-        <v>包子</v>
+        <v>猫</v>
       </c>
       <c r="C292" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9757,10 +9757,10 @@
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B293" t="str">
-        <v>菜</v>
+        <v>水</v>
       </c>
       <c r="C293" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9789,10 +9789,10 @@
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B294" t="str">
-        <v>茶</v>
+        <v>天</v>
       </c>
       <c r="C294" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9821,10 +9821,10 @@
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B295" t="str">
-        <v>饭</v>
+        <v>天气</v>
       </c>
       <c r="C295" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9853,10 +9853,10 @@
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B296" t="str">
-        <v>好吃</v>
+        <v>下雨</v>
       </c>
       <c r="C296" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9885,10 +9885,10 @@
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B297" t="str">
-        <v>鸡蛋</v>
+        <v>雪</v>
       </c>
       <c r="C297" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9917,10 +9917,10 @@
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B298" t="str">
-        <v>饺子</v>
+        <v>雨</v>
       </c>
       <c r="C298" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9949,10 +9949,10 @@
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>16. Đồ ăn &amp; Thức uống</v>
+        <v>15. Tự nhiên</v>
       </c>
       <c r="B299" t="str">
-        <v>米饭</v>
+        <v>早上</v>
       </c>
       <c r="C299" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -9984,7 +9984,7 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B300" t="str">
-        <v>面条儿</v>
+        <v>包子</v>
       </c>
       <c r="C300" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -10016,7 +10016,7 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B301" t="str">
-        <v>牛奶</v>
+        <v>菜</v>
       </c>
       <c r="C301" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -10048,7 +10048,7 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B302" t="str">
-        <v>苹果</v>
+        <v>茶</v>
       </c>
       <c r="C302" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -10080,7 +10080,7 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B303" t="str">
-        <v>水果</v>
+        <v>饭</v>
       </c>
       <c r="C303" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -10112,7 +10112,7 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B304" t="str">
-        <v>晚饭</v>
+        <v>好吃</v>
       </c>
       <c r="C304" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -10144,7 +10144,7 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B305" t="str">
-        <v>午饭</v>
+        <v>鸡蛋</v>
       </c>
       <c r="C305" t="str">
         <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
@@ -10176,182 +10176,470 @@
         <v>16. Đồ ăn &amp; Thức uống</v>
       </c>
       <c r="B306" t="str">
+        <v>饺子</v>
+      </c>
+      <c r="C306" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D306" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G306" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H306" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I306" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J306" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B307" t="str">
+        <v>米饭</v>
+      </c>
+      <c r="C307" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D307" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G307" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H307" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I307" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J307" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B308" t="str">
+        <v>面包</v>
+      </c>
+      <c r="C308" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D308" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G308" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H308" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I308" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J308" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B309" t="str">
+        <v>面条儿</v>
+      </c>
+      <c r="C309" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D309" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G309" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H309" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I309" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J309" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B310" t="str">
+        <v>牛奶</v>
+      </c>
+      <c r="C310" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D310" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E310" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F310" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G310" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H310" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I310" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J310" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B311" t="str">
+        <v>苹果</v>
+      </c>
+      <c r="C311" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D311" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E311" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F311" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G311" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H311" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I311" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J311" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B312" t="str">
+        <v>水果</v>
+      </c>
+      <c r="C312" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D312" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F312" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G312" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H312" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I312" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J312" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B313" t="str">
+        <v>晚饭</v>
+      </c>
+      <c r="C313" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D313" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F313" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G313" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H313" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I313" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J313" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B314" t="str">
+        <v>午饭</v>
+      </c>
+      <c r="C314" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D314" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F314" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G314" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H314" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I314" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J314" t="str">
+        <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>16. Đồ ăn &amp; Thức uống</v>
+      </c>
+      <c r="B315" t="str">
         <v>早饭</v>
       </c>
-      <c r="C306" t="str">
-        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
-      </c>
-      <c r="D306" t="str">
-        <v>HTML5, CSS3, JavaScript</v>
-      </c>
-      <c r="E306" t="str">
-        <v>Nhóm Phát triển HSK1</v>
-      </c>
-      <c r="F306" t="str">
-        <v>Board Game Trí Tuệ</v>
-      </c>
-      <c r="G306" t="str">
-        <v>index.html</v>
-      </c>
-      <c r="H306" t="str">
-        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
-      </c>
-      <c r="I306" t="str">
-        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
-      </c>
-      <c r="J306" t="str">
+      <c r="C315" t="str">
+        <v>HSK 1 - TRUY ĐUỔI KẺ TRỘM</v>
+      </c>
+      <c r="D315" t="str">
+        <v>HTML5, CSS3, JavaScript</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Nhóm Phát triển HSK1</v>
+      </c>
+      <c r="F315" t="str">
+        <v>Board Game Trí Tuệ</v>
+      </c>
+      <c r="G315" t="str">
+        <v>index.html</v>
+      </c>
+      <c r="H315" t="str">
+        <v>Ghi nhớ mặt chữ, ý nghĩa và cách phát âm từ vựng HSK 1 theo chủ đề thông qua trò chơi tương tác.</v>
+      </c>
+      <c r="I315" t="str">
+        <v>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</v>
+      </c>
+      <c r="J315" t="str">
         <v>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A2:A36"/>
-    <mergeCell ref="C2:C36"/>
-    <mergeCell ref="D2:D36"/>
-    <mergeCell ref="E2:E36"/>
-    <mergeCell ref="F2:F36"/>
-    <mergeCell ref="G2:G36"/>
-    <mergeCell ref="H2:H36"/>
-    <mergeCell ref="I2:I36"/>
-    <mergeCell ref="J2:J36"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="D37:D41"/>
-    <mergeCell ref="E37:E41"/>
-    <mergeCell ref="F37:F41"/>
-    <mergeCell ref="G37:G41"/>
-    <mergeCell ref="H37:H41"/>
-    <mergeCell ref="I37:I41"/>
-    <mergeCell ref="J37:J41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="G42:G45"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="I42:I45"/>
-    <mergeCell ref="J42:J45"/>
-    <mergeCell ref="A46:A62"/>
-    <mergeCell ref="C46:C62"/>
-    <mergeCell ref="D46:D62"/>
-    <mergeCell ref="E46:E62"/>
-    <mergeCell ref="F46:F62"/>
-    <mergeCell ref="G46:G62"/>
-    <mergeCell ref="H46:H62"/>
-    <mergeCell ref="I46:I62"/>
-    <mergeCell ref="J46:J62"/>
-    <mergeCell ref="A63:A80"/>
-    <mergeCell ref="C63:C80"/>
-    <mergeCell ref="D63:D80"/>
-    <mergeCell ref="E63:E80"/>
-    <mergeCell ref="F63:F80"/>
-    <mergeCell ref="G63:G80"/>
-    <mergeCell ref="H63:H80"/>
-    <mergeCell ref="I63:I80"/>
-    <mergeCell ref="J63:J80"/>
-    <mergeCell ref="A81:A100"/>
-    <mergeCell ref="C81:C100"/>
-    <mergeCell ref="D81:D100"/>
-    <mergeCell ref="E81:E100"/>
-    <mergeCell ref="F81:F100"/>
-    <mergeCell ref="G81:G100"/>
-    <mergeCell ref="H81:H100"/>
-    <mergeCell ref="I81:I100"/>
-    <mergeCell ref="J81:J100"/>
-    <mergeCell ref="A101:A128"/>
-    <mergeCell ref="C101:C128"/>
-    <mergeCell ref="D101:D128"/>
-    <mergeCell ref="E101:E128"/>
-    <mergeCell ref="F101:F128"/>
-    <mergeCell ref="G101:G128"/>
-    <mergeCell ref="H101:H128"/>
-    <mergeCell ref="I101:I128"/>
-    <mergeCell ref="J101:J128"/>
-    <mergeCell ref="A129:A138"/>
-    <mergeCell ref="C129:C138"/>
-    <mergeCell ref="D129:D138"/>
-    <mergeCell ref="E129:E138"/>
-    <mergeCell ref="F129:F138"/>
-    <mergeCell ref="G129:G138"/>
-    <mergeCell ref="H129:H138"/>
-    <mergeCell ref="I129:I138"/>
-    <mergeCell ref="J129:J138"/>
-    <mergeCell ref="A139:A152"/>
-    <mergeCell ref="C139:C152"/>
-    <mergeCell ref="D139:D152"/>
-    <mergeCell ref="E139:E152"/>
-    <mergeCell ref="F139:F152"/>
-    <mergeCell ref="G139:G152"/>
-    <mergeCell ref="H139:H152"/>
-    <mergeCell ref="I139:I152"/>
-    <mergeCell ref="J139:J152"/>
-    <mergeCell ref="A153:A177"/>
-    <mergeCell ref="C153:C177"/>
-    <mergeCell ref="D153:D177"/>
-    <mergeCell ref="E153:E177"/>
-    <mergeCell ref="F153:F177"/>
-    <mergeCell ref="G153:G177"/>
-    <mergeCell ref="H153:H177"/>
-    <mergeCell ref="I153:I177"/>
-    <mergeCell ref="J153:J177"/>
-    <mergeCell ref="A178:A191"/>
-    <mergeCell ref="C178:C191"/>
-    <mergeCell ref="D178:D191"/>
-    <mergeCell ref="E178:E191"/>
-    <mergeCell ref="F178:F191"/>
-    <mergeCell ref="G178:G191"/>
-    <mergeCell ref="H178:H191"/>
-    <mergeCell ref="I178:I191"/>
-    <mergeCell ref="J178:J191"/>
-    <mergeCell ref="A192:A210"/>
-    <mergeCell ref="C192:C210"/>
-    <mergeCell ref="D192:D210"/>
-    <mergeCell ref="E192:E210"/>
-    <mergeCell ref="F192:F210"/>
-    <mergeCell ref="G192:G210"/>
-    <mergeCell ref="H192:H210"/>
-    <mergeCell ref="I192:I210"/>
-    <mergeCell ref="J192:J210"/>
-    <mergeCell ref="A211:A245"/>
-    <mergeCell ref="C211:C245"/>
-    <mergeCell ref="D211:D245"/>
-    <mergeCell ref="E211:E245"/>
-    <mergeCell ref="F211:F245"/>
-    <mergeCell ref="G211:G245"/>
-    <mergeCell ref="H211:H245"/>
-    <mergeCell ref="I211:I245"/>
-    <mergeCell ref="J211:J245"/>
-    <mergeCell ref="A246:A283"/>
-    <mergeCell ref="C246:C283"/>
-    <mergeCell ref="D246:D283"/>
-    <mergeCell ref="E246:E283"/>
-    <mergeCell ref="F246:F283"/>
-    <mergeCell ref="G246:G283"/>
-    <mergeCell ref="H246:H283"/>
-    <mergeCell ref="I246:I283"/>
-    <mergeCell ref="J246:J283"/>
-    <mergeCell ref="A284:A291"/>
-    <mergeCell ref="C284:C291"/>
-    <mergeCell ref="D284:D291"/>
-    <mergeCell ref="E284:E291"/>
-    <mergeCell ref="F284:F291"/>
-    <mergeCell ref="G284:G291"/>
-    <mergeCell ref="H284:H291"/>
-    <mergeCell ref="I284:I291"/>
-    <mergeCell ref="J284:J291"/>
-    <mergeCell ref="A292:A306"/>
-    <mergeCell ref="C292:C306"/>
-    <mergeCell ref="D292:D306"/>
-    <mergeCell ref="E292:E306"/>
-    <mergeCell ref="F292:F306"/>
-    <mergeCell ref="G292:G306"/>
-    <mergeCell ref="H292:H306"/>
-    <mergeCell ref="I292:I306"/>
-    <mergeCell ref="J292:J306"/>
+    <mergeCell ref="A2:A37"/>
+    <mergeCell ref="C2:C37"/>
+    <mergeCell ref="D2:D37"/>
+    <mergeCell ref="E2:E37"/>
+    <mergeCell ref="F2:F37"/>
+    <mergeCell ref="G2:G37"/>
+    <mergeCell ref="H2:H37"/>
+    <mergeCell ref="I2:I37"/>
+    <mergeCell ref="J2:J37"/>
+    <mergeCell ref="A38:A42"/>
+    <mergeCell ref="C38:C42"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="E38:E42"/>
+    <mergeCell ref="F38:F42"/>
+    <mergeCell ref="G38:G42"/>
+    <mergeCell ref="H38:H42"/>
+    <mergeCell ref="I38:I42"/>
+    <mergeCell ref="J38:J42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="C43:C46"/>
+    <mergeCell ref="D43:D46"/>
+    <mergeCell ref="E43:E46"/>
+    <mergeCell ref="F43:F46"/>
+    <mergeCell ref="G43:G46"/>
+    <mergeCell ref="H43:H46"/>
+    <mergeCell ref="I43:I46"/>
+    <mergeCell ref="J43:J46"/>
+    <mergeCell ref="A47:A64"/>
+    <mergeCell ref="C47:C64"/>
+    <mergeCell ref="D47:D64"/>
+    <mergeCell ref="E47:E64"/>
+    <mergeCell ref="F47:F64"/>
+    <mergeCell ref="G47:G64"/>
+    <mergeCell ref="H47:H64"/>
+    <mergeCell ref="I47:I64"/>
+    <mergeCell ref="J47:J64"/>
+    <mergeCell ref="A65:A84"/>
+    <mergeCell ref="C65:C84"/>
+    <mergeCell ref="D65:D84"/>
+    <mergeCell ref="E65:E84"/>
+    <mergeCell ref="F65:F84"/>
+    <mergeCell ref="G65:G84"/>
+    <mergeCell ref="H65:H84"/>
+    <mergeCell ref="I65:I84"/>
+    <mergeCell ref="J65:J84"/>
+    <mergeCell ref="A85:A104"/>
+    <mergeCell ref="C85:C104"/>
+    <mergeCell ref="D85:D104"/>
+    <mergeCell ref="E85:E104"/>
+    <mergeCell ref="F85:F104"/>
+    <mergeCell ref="G85:G104"/>
+    <mergeCell ref="H85:H104"/>
+    <mergeCell ref="I85:I104"/>
+    <mergeCell ref="J85:J104"/>
+    <mergeCell ref="A105:A131"/>
+    <mergeCell ref="C105:C131"/>
+    <mergeCell ref="D105:D131"/>
+    <mergeCell ref="E105:E131"/>
+    <mergeCell ref="F105:F131"/>
+    <mergeCell ref="G105:G131"/>
+    <mergeCell ref="H105:H131"/>
+    <mergeCell ref="I105:I131"/>
+    <mergeCell ref="J105:J131"/>
+    <mergeCell ref="A132:A141"/>
+    <mergeCell ref="C132:C141"/>
+    <mergeCell ref="D132:D141"/>
+    <mergeCell ref="E132:E141"/>
+    <mergeCell ref="F132:F141"/>
+    <mergeCell ref="G132:G141"/>
+    <mergeCell ref="H132:H141"/>
+    <mergeCell ref="I132:I141"/>
+    <mergeCell ref="J132:J141"/>
+    <mergeCell ref="A142:A155"/>
+    <mergeCell ref="C142:C155"/>
+    <mergeCell ref="D142:D155"/>
+    <mergeCell ref="E142:E155"/>
+    <mergeCell ref="F142:F155"/>
+    <mergeCell ref="G142:G155"/>
+    <mergeCell ref="H142:H155"/>
+    <mergeCell ref="I142:I155"/>
+    <mergeCell ref="J142:J155"/>
+    <mergeCell ref="A156:A181"/>
+    <mergeCell ref="C156:C181"/>
+    <mergeCell ref="D156:D181"/>
+    <mergeCell ref="E156:E181"/>
+    <mergeCell ref="F156:F181"/>
+    <mergeCell ref="G156:G181"/>
+    <mergeCell ref="H156:H181"/>
+    <mergeCell ref="I156:I181"/>
+    <mergeCell ref="J156:J181"/>
+    <mergeCell ref="A182:A196"/>
+    <mergeCell ref="C182:C196"/>
+    <mergeCell ref="D182:D196"/>
+    <mergeCell ref="E182:E196"/>
+    <mergeCell ref="F182:F196"/>
+    <mergeCell ref="G182:G196"/>
+    <mergeCell ref="H182:H196"/>
+    <mergeCell ref="I182:I196"/>
+    <mergeCell ref="J182:J196"/>
+    <mergeCell ref="A197:A215"/>
+    <mergeCell ref="C197:C215"/>
+    <mergeCell ref="D197:D215"/>
+    <mergeCell ref="E197:E215"/>
+    <mergeCell ref="F197:F215"/>
+    <mergeCell ref="G197:G215"/>
+    <mergeCell ref="H197:H215"/>
+    <mergeCell ref="I197:I215"/>
+    <mergeCell ref="J197:J215"/>
+    <mergeCell ref="A216:A250"/>
+    <mergeCell ref="C216:C250"/>
+    <mergeCell ref="D216:D250"/>
+    <mergeCell ref="E216:E250"/>
+    <mergeCell ref="F216:F250"/>
+    <mergeCell ref="G216:G250"/>
+    <mergeCell ref="H216:H250"/>
+    <mergeCell ref="I216:I250"/>
+    <mergeCell ref="J216:J250"/>
+    <mergeCell ref="A251:A290"/>
+    <mergeCell ref="C251:C290"/>
+    <mergeCell ref="D251:D290"/>
+    <mergeCell ref="E251:E290"/>
+    <mergeCell ref="F251:F290"/>
+    <mergeCell ref="G251:G290"/>
+    <mergeCell ref="H251:H290"/>
+    <mergeCell ref="I251:I290"/>
+    <mergeCell ref="J251:J290"/>
+    <mergeCell ref="A291:A299"/>
+    <mergeCell ref="C291:C299"/>
+    <mergeCell ref="D291:D299"/>
+    <mergeCell ref="E291:E299"/>
+    <mergeCell ref="F291:F299"/>
+    <mergeCell ref="G291:G299"/>
+    <mergeCell ref="H291:H299"/>
+    <mergeCell ref="I291:I299"/>
+    <mergeCell ref="J291:J299"/>
+    <mergeCell ref="A300:A315"/>
+    <mergeCell ref="C300:C315"/>
+    <mergeCell ref="D300:D315"/>
+    <mergeCell ref="E300:E315"/>
+    <mergeCell ref="F300:F315"/>
+    <mergeCell ref="G300:G315"/>
+    <mergeCell ref="H300:H315"/>
+    <mergeCell ref="I300:I315"/>
+    <mergeCell ref="J300:J315"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J306"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J315"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>